<commit_message>
seperat enemy data + killQuests + start on rewards
</commit_message>
<xml_diff>
--- a/Benchmark Feature List.xlsx
+++ b/Benchmark Feature List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaron\Desktop\Study\2e Year\SoftwareArchitecture\Software_Achitecture_Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBD7392C-4E4B-48CD-82B7-ADAAED457CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{721AF26D-ACF3-4846-A35A-45A59C2D974F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{DFC97FD2-4022-1548-A7B7-2F9FA8F56567}"/>
   </bookViews>
@@ -163,7 +163,7 @@
     <t>Normal</t>
   </si>
   <si>
-    <t>50% done</t>
+    <t>High</t>
   </si>
 </sst>
 </file>
@@ -322,7 +322,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -663,7 +663,7 @@
     <col min="1" max="1" width="164.25" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.4140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.08203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="5" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.5" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
@@ -693,7 +693,7 @@
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
     </row>
-    <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -702,7 +702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="31" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
@@ -712,8 +712,8 @@
       <c r="C5" s="13" t="b">
         <v>0</v>
       </c>
-      <c r="D5" s="14" t="s">
-        <v>41</v>
+      <c r="D5" s="14">
+        <v>0.5</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -726,6 +726,9 @@
       <c r="C6" s="13" t="b">
         <v>0</v>
       </c>
+      <c r="D6" s="14">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
@@ -733,30 +736,28 @@
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6"/>
       <c r="B8" s="3"/>
-      <c r="C8" s="13" t="b">
-        <v>0</v>
-      </c>
+      <c r="C8" s="5"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>30</v>
       </c>
       <c r="B9" s="4"/>
-      <c r="C9" s="13" t="b">
-        <v>0</v>
-      </c>
+      <c r="C9" s="5"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="5"/>
+      <c r="B10" s="5" t="s">
+        <v>41</v>
+      </c>
       <c r="C10" s="13" t="b">
         <v>0</v>
       </c>

</xml_diff>